<commit_message>
chloride var selection table
</commit_message>
<xml_diff>
--- a/Benchmarks/Water Chemistry/Chloride/Chloride_Var selection decisions.xlsx
+++ b/Benchmarks/Water Chemistry/Chloride/Chloride_Var selection decisions.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/sabine_berzins_deq_oregon_gov/Documents/Documents/BioMonORDEQ/Benchmarks/Water Chemistry/Chloride/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/adam_thompson_deq_oregon_gov/Documents/Documents/BioMonORDEQ/Benchmarks/Water Chemistry/Chloride/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{CDC6F8B2-D72D-412E-9686-4A4B80E69C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78BEF76F-DF47-49FF-BF2F-33FB10CFF37B}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{CDC6F8B2-D72D-412E-9686-4A4B80E69C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E16C3B76-DF95-4EC5-A4C4-E23C71EA1847}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30624" yWindow="0" windowWidth="15552" windowHeight="16656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$132</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="151">
   <si>
     <t>num_vars</t>
   </si>
@@ -441,9 +441,6 @@
     <t>Keep or Remove</t>
   </si>
   <si>
-    <t>TEXTJOIN(", ", TRUE, A:A)</t>
-  </si>
-  <si>
     <t>REMOVE</t>
   </si>
   <si>
@@ -451,6 +448,48 @@
   </si>
   <si>
     <t>distance</t>
+  </si>
+  <si>
+    <t>have other kffact</t>
+  </si>
+  <si>
+    <t>KEEP</t>
+  </si>
+  <si>
+    <t>kept bfi</t>
+  </si>
+  <si>
+    <t>kept calcium</t>
+  </si>
+  <si>
+    <t>correlated with mixed forest, winter stream temps, and elev but keeping for interest sake</t>
+  </si>
+  <si>
+    <t>straightline distance to coast polygon</t>
+  </si>
+  <si>
+    <t>kept ammonia</t>
+  </si>
+  <si>
+    <t>more encompassing</t>
+  </si>
+  <si>
+    <t>kept % erod</t>
+  </si>
+  <si>
+    <t>kept burn area</t>
+  </si>
+  <si>
+    <t>corr with distance but keep anyway</t>
+  </si>
+  <si>
+    <t>better spread b/t hi and lo</t>
+  </si>
+  <si>
+    <t>better CV than others</t>
+  </si>
+  <si>
+    <t>kept precip-evt</t>
   </si>
 </sst>
 </file>
@@ -846,16 +885,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D132"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="59.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="59.6328125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -869,738 +909,1044 @@
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" t="s">
         <v>135</v>
       </c>
-      <c r="C11" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
+      <c r="B13" t="s">
+        <v>138</v>
+      </c>
       <c r="D13" s="7"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>13</v>
       </c>
+      <c r="B14" t="s">
+        <v>134</v>
+      </c>
       <c r="D14" s="7"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
+      <c r="B15" t="s">
+        <v>134</v>
+      </c>
       <c r="D15" s="7"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>134</v>
+      </c>
+      <c r="C26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>30</v>
       </c>
+      <c r="B31" t="s">
+        <v>134</v>
+      </c>
       <c r="D31" s="9"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>31</v>
       </c>
+      <c r="B32" t="s">
+        <v>134</v>
+      </c>
       <c r="D32" s="9"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>32</v>
       </c>
+      <c r="B33" t="s">
+        <v>134</v>
+      </c>
       <c r="D33" s="9"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>134</v>
+      </c>
+      <c r="C37" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D40" s="7"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>40</v>
       </c>
       <c r="D41" s="7"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>41</v>
       </c>
+      <c r="B42" t="s">
+        <v>134</v>
+      </c>
       <c r="D42" s="7"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>138</v>
+      </c>
+      <c r="C43" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D44" s="7"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>44</v>
       </c>
+      <c r="B45" t="s">
+        <v>134</v>
+      </c>
       <c r="D45" s="7"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>45</v>
       </c>
+      <c r="B46" t="s">
+        <v>138</v>
+      </c>
       <c r="D46" s="7"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>134</v>
+      </c>
+      <c r="C52" t="s">
         <v>135</v>
       </c>
-      <c r="C52" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>56</v>
       </c>
       <c r="B57" t="s">
+        <v>134</v>
+      </c>
+      <c r="C57" t="s">
         <v>135</v>
       </c>
-      <c r="C57" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
+        <v>134</v>
+      </c>
+      <c r="C60" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D62" s="7"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D63" s="7"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>134</v>
+      </c>
+      <c r="C64" t="s">
         <v>135</v>
       </c>
-      <c r="C64" t="s">
-        <v>136</v>
-      </c>
       <c r="D64" s="7"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>64</v>
       </c>
       <c r="D65" s="7"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>134</v>
+      </c>
+      <c r="C66" t="s">
         <v>135</v>
       </c>
-      <c r="C66" t="s">
-        <v>136</v>
-      </c>
       <c r="D66" s="7"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>134</v>
+      </c>
+      <c r="C70" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
         <v>70</v>
       </c>
       <c r="B71" t="s">
+        <v>134</v>
+      </c>
+      <c r="C71" t="s">
         <v>135</v>
       </c>
-      <c r="C71" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B73" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B74" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B75" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B77" t="s">
+        <v>134</v>
+      </c>
+      <c r="C77" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B78" t="s">
+        <v>134</v>
+      </c>
+      <c r="C78" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B79" t="s">
+        <v>138</v>
+      </c>
+      <c r="C79" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B81" t="s">
+        <v>134</v>
+      </c>
+      <c r="C81" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
         <v>81</v>
       </c>
       <c r="B82" t="s">
+        <v>134</v>
+      </c>
+      <c r="C82" t="s">
         <v>135</v>
       </c>
-      <c r="C82" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B86" t="s">
+        <v>134</v>
+      </c>
+      <c r="C86" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B87" t="s">
+        <v>134</v>
+      </c>
+      <c r="C87" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B89" t="s">
+        <v>138</v>
+      </c>
+      <c r="C89" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B90" t="s">
+        <v>134</v>
+      </c>
+      <c r="C90" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B94" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B96" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B97" t="s">
+        <v>138</v>
+      </c>
+      <c r="C97" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
         <v>97</v>
       </c>
+      <c r="B98" t="s">
+        <v>134</v>
+      </c>
+      <c r="C98" t="s">
+        <v>150</v>
+      </c>
       <c r="D98" s="7"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
         <v>98</v>
       </c>
+      <c r="B99" t="s">
+        <v>134</v>
+      </c>
+      <c r="C99" t="s">
+        <v>150</v>
+      </c>
       <c r="D99" s="7"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
         <v>99</v>
       </c>
+      <c r="B100" t="s">
+        <v>134</v>
+      </c>
+      <c r="C100" t="s">
+        <v>150</v>
+      </c>
       <c r="D100" s="7"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
         <v>101</v>
       </c>
       <c r="D102" s="8"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D103" s="8"/>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
         <v>103</v>
       </c>
       <c r="D104" s="8"/>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B106" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B109" t="s">
+        <v>134</v>
+      </c>
+      <c r="C109" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B110" t="s">
+        <v>134</v>
+      </c>
+      <c r="C110" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B113" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B115" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="s">
         <v>115</v>
       </c>
+      <c r="B116" t="s">
+        <v>134</v>
+      </c>
       <c r="D116" s="7"/>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="B117" t="s">
+        <v>138</v>
+      </c>
       <c r="D117" s="7"/>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
         <v>117</v>
       </c>
+      <c r="B118" t="s">
+        <v>134</v>
+      </c>
       <c r="D118" s="7"/>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
         <v>118</v>
       </c>
+      <c r="B119" t="s">
+        <v>134</v>
+      </c>
+      <c r="C119" t="s">
+        <v>139</v>
+      </c>
       <c r="D119" s="7"/>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
         <v>119</v>
       </c>
+      <c r="B120" t="s">
+        <v>134</v>
+      </c>
+      <c r="C120" t="s">
+        <v>139</v>
+      </c>
       <c r="D120" s="7"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
         <v>120</v>
       </c>
+      <c r="B121" t="s">
+        <v>134</v>
+      </c>
+      <c r="C121" t="s">
+        <v>139</v>
+      </c>
       <c r="D121" s="7"/>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
         <v>121</v>
       </c>
+      <c r="B122" t="s">
+        <v>134</v>
+      </c>
+      <c r="C122" t="s">
+        <v>139</v>
+      </c>
       <c r="D122" s="7"/>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B124" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B125" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B127" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="B129" t="s">
+        <v>138</v>
+      </c>
       <c r="D129" s="7"/>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
         <v>129</v>
       </c>
       <c r="D130" s="7"/>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
         <v>130</v>
       </c>
+      <c r="B131" t="s">
+        <v>134</v>
+      </c>
       <c r="D131" s="7"/>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="B132" t="s">
+        <v>138</v>
+      </c>
+      <c r="C132" t="s">
+        <v>141</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D131" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D132" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters blank="1">
+        <filter val="KEEP"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="9">
     <mergeCell ref="D13:D15"/>
     <mergeCell ref="D62:D66"/>
@@ -1612,7 +1958,7 @@
     <mergeCell ref="D40:D42"/>
     <mergeCell ref="D31:D33"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2:B131">
+  <conditionalFormatting sqref="B2:B132">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"KEEP"</formula>
     </cfRule>
@@ -1621,7 +1967,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B131" xr:uid="{EB42C186-6836-4773-A6E5-B88EA86420AD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B132" xr:uid="{EB42C186-6836-4773-A6E5-B88EA86420AD}">
       <formula1>"KEEP, REMOVE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1631,12 +1977,376 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{436B77FA-BCAA-44EA-8D79-399215CFE77B}">
-  <dimension ref="C1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C73"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C1" t="s">
-        <v>134</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="str">
+        <f>_xlfn.TEXTJOIN(", ", TRUE, A:A)</f>
+        <v>BFIWS, CANALDENSWS, CAOWS, CLAYWS, COMPSTRGTHWS, DAMDENSWS, ELEVWS, FERTWS, HYDRLCONDWS, KFFACTWS, MINEDENSWS, MSST2008, NA2OWS, NANIWS, NH42008WS, NHD_pSLOPE, NPDESDENSWS, NWS, OMWS, PCT_EROD, PCTAGDRAINAGEWS, PCTAGSLPMID2001WS, PCTALKINTRUVOLWS, PCTALLUVCOASTWS, PCTBL2001WS, PCTBURNAREA2002WS, PCTCARBRESIDWS, PCTCOLLUVSEDWS, PCTCONIF2001WS, PCTCROP2001WS, PCTDECID2001WS, PCTEOLFINEWS, PCTEXTRUVOLWS, PCTFRSTLOSS2002WS, PCTGLACLAKECRSWS, PCTGLACLAKEFINEWS, PCTGLACTILCRSWS, PCTGRS2001WS, PCTHBWET2001WS, PCTICE2001WS, PCTIMP2001WS, PCTINCVEGRESP2002WS, PCTMXFST2001WS, PCTNONAGINTRODMANAGVEGWS, PCTOW2001WS, PCTSALLAKEWS, PCTSHRB2001WS, PCTURBHI2001WS, PCTURBLO2001WS, PCTURBOP2001WS, PCTWATERWS, PCTWDWET2001WS, PESTIC1997WS, POPDEN2010WS, PRECIP_MINUS_EVTWS, RCKDEPWS, RDCRSSLPWTDWS, RDCRSWS, RDDENSWS, ROCKNWS, RUNOFFWS, SANDWS, SEPTICWS, STRMPOW_CAT, SUPERFUNDDENSWS, SWS, TMAX9120WS, TRIDENSWS, WETINDEXWS, WTDEPWS, WWTPALLDENSWS, WWTPMAJORDENSWS, distance</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A53" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" s="5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" s="5" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>